<commit_message>
TGS.Ol CHE, STD + Excel
</commit_message>
<xml_diff>
--- a/data/obx_xlsx/TGS.OL.xlsx
+++ b/data/obx_xlsx/TGS.OL.xlsx
@@ -10538,8 +10538,14 @@
       <c r="O29" s="16">
         <v>2006.4</v>
       </c>
-      <c r="P29" s="15"/>
-      <c r="Q29" s="15"/>
+      <c r="P29" s="15">
+        <f t="shared" ref="P29:Q29" si="1">P30+P32</f>
+        <v>1689.4</v>
+      </c>
+      <c r="Q29" s="15">
+        <f t="shared" si="1"/>
+        <v>1410.65</v>
+      </c>
       <c r="R29" s="16">
         <v>1030.03</v>
       </c>
@@ -12162,55 +12168,55 @@
         <v>9681.28</v>
       </c>
       <c r="C68" s="20">
-        <f t="shared" ref="C68:O68" si="1">SUM(C69,C73)</f>
+        <f t="shared" ref="C68:O68" si="2">SUM(C69,C73)</f>
         <v>1337.53</v>
       </c>
       <c r="D68" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1421.46</v>
       </c>
       <c r="E68" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>171.9</v>
       </c>
       <c r="F68" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>236.8</v>
       </c>
       <c r="G68" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>216.91</v>
       </c>
       <c r="H68" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>197.19</v>
       </c>
       <c r="I68" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>161.39</v>
       </c>
       <c r="J68" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>198.84</v>
       </c>
       <c r="K68" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>266.81</v>
       </c>
       <c r="L68" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>322.61</v>
       </c>
       <c r="M68" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>320.3</v>
       </c>
       <c r="N68" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>178.15</v>
       </c>
       <c r="O68" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>116.92</v>
       </c>
       <c r="P68" s="20">

</xml_diff>